<commit_message>
update: add Mutton Biryani and Beerakaya milk recipes
</commit_message>
<xml_diff>
--- a/br-pr-family-recipe-book.xlsx
+++ b/br-pr-family-recipe-book.xlsx
@@ -11,14 +11,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId7" roundtripDataChecksum="Uhn/OAMKfNOb0qC8AGXE/Q6VgqMq+2PFtKuJWpZAyhE="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId7" roundtripDataChecksum="3UgsNuseQT/20hM5LY+LitwbEFJDANKWSU8A6xLlLsw="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="107">
   <si>
     <t>📖  Family Recipe Book</t>
   </si>
@@ -44,6 +44,12 @@
     <t>recipe 6</t>
   </si>
   <si>
+    <t>recipe 7</t>
+  </si>
+  <si>
+    <t>recipe 8</t>
+  </si>
+  <si>
     <t>id</t>
   </si>
   <si>
@@ -65,6 +71,25 @@
     <t>Saggu Biyyam</t>
   </si>
   <si>
+    <t>Mutton Biryani</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beerakaya milk
+</t>
+  </si>
+  <si>
+    <t>mango pappu</t>
+  </si>
+  <si>
+    <t>Mysoore Bonda</t>
+  </si>
+  <si>
+    <t>Punugu</t>
+  </si>
+  <si>
+    <t>pala thalikalu</t>
+  </si>
+  <si>
     <t>emoji</t>
   </si>
   <si>
@@ -80,10 +105,16 @@
     <t>weekend</t>
   </si>
   <si>
-    <t>daily</t>
-  </si>
-  <si>
-    <t>daily / weekend / special / festival</t>
+    <t>weekly twice</t>
+  </si>
+  <si>
+    <t>Festive, friends gathering</t>
+  </si>
+  <si>
+    <t>Daily</t>
+  </si>
+  <si>
+    <t>weekly</t>
   </si>
   <si>
     <t>time</t>
@@ -98,6 +129,12 @@
     <t>30 mins</t>
   </si>
   <si>
+    <t>30min</t>
+  </si>
+  <si>
+    <t>1 hr</t>
+  </si>
+  <si>
     <t>servings</t>
   </si>
   <si>
@@ -107,6 +144,9 @@
     <t>4 people</t>
   </si>
   <si>
+    <t>4-10 people</t>
+  </si>
+  <si>
     <t>ingredients</t>
   </si>
   <si>
@@ -117,6 +157,18 @@
   </si>
   <si>
     <t>Saggu biyyam, water, milk Jaggery</t>
+  </si>
+  <si>
+    <t>basmati rice, mutton, yogurt, onion, ginger-garlic paste, biryani masala, saffron milk, ghee, mint leaves, fried onions, whole spices</t>
+  </si>
+  <si>
+    <t>onions, beerakaya</t>
+  </si>
+  <si>
+    <t>Yougurt, Maida, oil, onions, mirchi</t>
+  </si>
+  <si>
+    <t>Idly batter, upma ravva, maida, onions, mirchi, cooriander</t>
   </si>
   <si>
     <t>steps</t>
@@ -150,6 +202,32 @@
 That's it and serve it with love to your family</t>
   </si>
   <si>
+    <t>Marinate mutton in yogurt and spices for at least 1 hour.
+it's better presuure cook mutton (light boiled)
+Soak basmati rice 30 mins, par-boil until 70% cooked.
+Fry onions until deep golden and crispy.
+Layer chicken at bottom of heavy pot.
+Add par-cooked rice, fried onions, mint on top.
+Drizzle saffron milk and ghee.
+Seal tightly and cook dum on very low heat 30 mins.
+Gently mix from bottom and serve with raita.</t>
+  </si>
+  <si>
+    <t>cut beerakaya small pieces peel the skin off
+fry everything until get to a fried state
+mix milk and keep it on the stove for a bit</t>
+  </si>
+  <si>
+    <t>Soak maida, salt, yogurt prior night
+Oil to the fry temperature
+Fry the maida soaked in oil
+use baking soda for fluffy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Make sure you have idly batter fermented
+mix idly better with upma ravva (little bit), </t>
+  </si>
+  <si>
     <t>notes</t>
   </si>
   <si>
@@ -162,7 +240,13 @@
     <t>added_by</t>
   </si>
   <si>
-    <t>Mom</t>
+    <t>Raji</t>
+  </si>
+  <si>
+    <t>Raja's mom</t>
+  </si>
+  <si>
+    <t>Raji's mom</t>
   </si>
   <si>
     <t>date_added</t>
@@ -205,6 +289,9 @@
   </si>
   <si>
     <t>frequency</t>
+  </si>
+  <si>
+    <t>daily</t>
   </si>
   <si>
     <t>saturday</t>
@@ -292,7 +379,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -320,12 +407,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11.0"/>
-      <color rgb="FFAAAAAA"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
       <sz val="10.0"/>
       <color rgb="FF2D4A3E"/>
       <name val="Arial"/>
@@ -334,6 +415,11 @@
       <sz val="10.0"/>
       <color rgb="FF333333"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <i/>
@@ -351,6 +437,12 @@
       <b/>
       <sz val="10.0"/>
       <color rgb="FF155724"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11.0"/>
+      <color rgb="FFAAAAAA"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -408,12 +500,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF4A6B5E"/>
-        <bgColor rgb="FF4A6B5E"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFF0F4F2"/>
         <bgColor rgb="FFF0F4F2"/>
       </patternFill>
@@ -450,12 +536,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF4A6B5E"/>
+        <bgColor rgb="FF4A6B5E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFF3CD"/>
         <bgColor rgb="FFFFF3CD"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="5">
     <border/>
     <border>
       <left/>
@@ -463,11 +555,6 @@
       <bottom/>
     </border>
     <border>
-      <top/>
-      <bottom/>
-    </border>
-    <border>
-      <right/>
       <top/>
       <bottom/>
     </border>
@@ -511,74 +598,76 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="3" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="5" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="3" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="3" fillId="5" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf borderId="3" fillId="6" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="7" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="6" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="7" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="8" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf borderId="3" fillId="9" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="10" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="11" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="6" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf borderId="4" fillId="7" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="8" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="5" fillId="9" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf borderId="4" fillId="10" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="11" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="5" fillId="9" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf borderId="4" fillId="7" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="8" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="6" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="3" fillId="5" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="8" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="3" fillId="7" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="7" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="3" fillId="6" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="9" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="8" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="11" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="3" fillId="10" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="10" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="3" fillId="9" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="8" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="7" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="8" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="7" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="12" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="12" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="11" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="10" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -804,8 +893,11 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="16.0"/>
     <col customWidth="1" min="2" max="3" width="38.0"/>
-    <col customWidth="1" min="4" max="6" width="32.0"/>
-    <col customWidth="1" min="7" max="25" width="8.71"/>
+    <col customWidth="1" min="4" max="7" width="32.0"/>
+    <col customWidth="1" min="8" max="8" width="27.57"/>
+    <col customWidth="1" min="9" max="9" width="25.29"/>
+    <col customWidth="1" min="10" max="10" width="29.57"/>
+    <col customWidth="1" min="11" max="26" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="36.0" customHeight="1">
@@ -814,214 +906,328 @@
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
-      <c r="D1" s="3"/>
+      <c r="D1" s="2"/>
     </row>
     <row r="2" ht="21.75" customHeight="1">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="3"/>
+      <c r="D2" s="2"/>
     </row>
     <row r="3" ht="6.0" customHeight="1"/>
     <row r="4" ht="27.75" customHeight="1">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="5" t="s">
         <v>7</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="5" ht="21.75" customHeight="1">
-      <c r="A5" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="9" t="s">
+      <c r="A5" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="9">
+      <c r="B5" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="8">
         <v>1004.0</v>
       </c>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
+      <c r="E5" s="9">
+        <v>1005.0</v>
+      </c>
+      <c r="F5" s="8">
+        <v>1105.0</v>
+      </c>
+      <c r="G5" s="10">
+        <v>1106.0</v>
+      </c>
+      <c r="H5" s="10">
+        <v>1107.0</v>
+      </c>
+      <c r="I5" s="11">
+        <v>1108.0</v>
+      </c>
+      <c r="J5" s="11">
+        <v>1109.0</v>
+      </c>
     </row>
     <row r="6" ht="21.75" customHeight="1">
-      <c r="A6" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="9" t="s">
+      <c r="A6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="B6" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
+      <c r="C6" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="J6" s="11" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="7" ht="21.75" customHeight="1">
-      <c r="A7" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
+      <c r="A7" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="12"/>
+      <c r="E7" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="F7" s="12"/>
+      <c r="G7" s="12"/>
     </row>
     <row r="8" ht="21.75" customHeight="1">
-      <c r="A8" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>19</v>
+      <c r="A8" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>29</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="F8" s="13" t="s">
-        <v>21</v>
+        <v>27</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="H8" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="I8" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="J8" s="11" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="9" ht="21.75" customHeight="1">
-      <c r="A9" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
+      <c r="A9" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="10" ht="21.75" customHeight="1">
-      <c r="A10" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
+      <c r="A10" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="H10" s="11" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="11" ht="39.75" customHeight="1">
-      <c r="A11" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
+      <c r="A11" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H11" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="I11" s="11" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="12" ht="120.0" customHeight="1">
-      <c r="A12" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
+      <c r="A12" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="H12" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="I12" s="11" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="13" ht="34.5" customHeight="1">
-      <c r="A13" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="D13" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
+      <c r="A13" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F13" s="12"/>
+      <c r="G13" s="12"/>
     </row>
     <row r="14" ht="21.75" customHeight="1">
-      <c r="A14" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="B14" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="C14" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="D14" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
+      <c r="A14" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="F14" s="12"/>
+      <c r="G14" s="12"/>
     </row>
     <row r="15" ht="21.75" customHeight="1">
-      <c r="A15" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="D15" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
+      <c r="A15" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -2005,8 +2211,8 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
@@ -2030,126 +2236,126 @@
   <sheetData>
     <row r="1" ht="36.0" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
-      <c r="D1" s="3"/>
+      <c r="D1" s="2"/>
     </row>
     <row r="2" ht="21.75" customHeight="1">
-      <c r="A2" s="4" t="s">
-        <v>45</v>
+      <c r="A2" s="3" t="s">
+        <v>68</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="3"/>
+      <c r="D2" s="2"/>
     </row>
     <row r="3" ht="6.0" customHeight="1"/>
     <row r="4" ht="27.75" customHeight="1">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>49</v>
+      <c r="B4" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="5" ht="21.75" customHeight="1">
       <c r="A5" s="16" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="D5" s="19"/>
       <c r="E5" s="19"/>
     </row>
     <row r="6" ht="21.75" customHeight="1">
       <c r="A6" s="16" t="s">
-        <v>52</v>
+        <v>75</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D6" s="19"/>
       <c r="E6" s="19"/>
     </row>
     <row r="7" ht="21.75" customHeight="1">
       <c r="A7" s="16" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>54</v>
+        <v>77</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="D7" s="19"/>
       <c r="E7" s="19"/>
     </row>
     <row r="8" ht="21.75" customHeight="1">
       <c r="A8" s="16" t="s">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>20</v>
+        <v>79</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>57</v>
+        <v>81</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>57</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" ht="21.75" customHeight="1">
       <c r="A9" s="16" t="s">
-        <v>58</v>
+        <v>82</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>59</v>
+        <v>83</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>60</v>
+        <v>84</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" ht="21.75" customHeight="1">
       <c r="A10" s="16" t="s">
-        <v>62</v>
+        <v>86</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>63</v>
+        <v>87</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>63</v>
+        <v>87</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -3157,165 +3363,165 @@
   <sheetData>
     <row r="1" ht="39.75" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
-      <c r="D1" s="3"/>
+      <c r="D1" s="2"/>
     </row>
     <row r="2" ht="7.5" customHeight="1">
       <c r="A2" s="22"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="3"/>
+      <c r="D2" s="2"/>
     </row>
     <row r="3" ht="24.0" customHeight="1">
       <c r="A3" s="23" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
-      <c r="D3" s="3"/>
+      <c r="D3" s="2"/>
     </row>
     <row r="4" ht="19.5" customHeight="1">
       <c r="A4" s="24" t="s">
-        <v>67</v>
+        <v>91</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
-      <c r="D4" s="3"/>
+      <c r="D4" s="2"/>
     </row>
     <row r="5" ht="19.5" customHeight="1">
       <c r="A5" s="24" t="s">
-        <v>68</v>
+        <v>92</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="3"/>
+      <c r="D5" s="2"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
       <c r="A6" s="24" t="s">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="3"/>
+      <c r="D6" s="2"/>
     </row>
     <row r="7" ht="19.5" customHeight="1">
       <c r="A7" s="24" t="s">
-        <v>70</v>
+        <v>94</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="3"/>
+      <c r="D7" s="2"/>
     </row>
     <row r="8" ht="19.5" customHeight="1">
       <c r="A8" s="24" t="s">
-        <v>71</v>
+        <v>95</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
-      <c r="D8" s="3"/>
+      <c r="D8" s="2"/>
     </row>
     <row r="9" ht="19.5" customHeight="1">
       <c r="A9" s="25" t="s">
-        <v>72</v>
+        <v>96</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
-      <c r="D9" s="3"/>
+      <c r="D9" s="2"/>
     </row>
     <row r="10" ht="7.5" customHeight="1">
       <c r="A10" s="22"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
-      <c r="D10" s="3"/>
+      <c r="D10" s="2"/>
     </row>
     <row r="11" ht="24.0" customHeight="1">
       <c r="A11" s="23" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
-      <c r="D11" s="3"/>
+      <c r="D11" s="2"/>
     </row>
     <row r="12" ht="19.5" customHeight="1">
       <c r="A12" s="24" t="s">
-        <v>74</v>
+        <v>98</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
-      <c r="D12" s="3"/>
+      <c r="D12" s="2"/>
     </row>
     <row r="13" ht="19.5" customHeight="1">
       <c r="A13" s="24" t="s">
-        <v>75</v>
+        <v>99</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
-      <c r="D13" s="3"/>
+      <c r="D13" s="2"/>
     </row>
     <row r="14" ht="19.5" customHeight="1">
       <c r="A14" s="24" t="s">
-        <v>76</v>
+        <v>100</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
-      <c r="D14" s="3"/>
+      <c r="D14" s="2"/>
     </row>
     <row r="15" ht="19.5" customHeight="1">
       <c r="A15" s="24" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
-      <c r="D15" s="3"/>
+      <c r="D15" s="2"/>
     </row>
     <row r="16" ht="7.5" customHeight="1">
       <c r="A16" s="22"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
-      <c r="D16" s="3"/>
+      <c r="D16" s="2"/>
     </row>
     <row r="17" ht="24.0" customHeight="1">
       <c r="A17" s="23" t="s">
-        <v>78</v>
+        <v>102</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
-      <c r="D17" s="3"/>
+      <c r="D17" s="2"/>
     </row>
     <row r="18" ht="19.5" customHeight="1">
       <c r="A18" s="24" t="s">
-        <v>79</v>
+        <v>103</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
-      <c r="D18" s="3"/>
+      <c r="D18" s="2"/>
     </row>
     <row r="19" ht="19.5" customHeight="1">
       <c r="A19" s="24" t="s">
-        <v>80</v>
+        <v>104</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
-      <c r="D19" s="3"/>
+      <c r="D19" s="2"/>
     </row>
     <row r="20" ht="19.5" customHeight="1">
       <c r="A20" s="24" t="s">
-        <v>81</v>
+        <v>105</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
-      <c r="D20" s="3"/>
+      <c r="D20" s="2"/>
     </row>
     <row r="21" ht="19.5" customHeight="1">
       <c r="A21" s="26" t="s">
-        <v>82</v>
+        <v>106</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
-      <c r="D21" s="3"/>
+      <c r="D21" s="2"/>
     </row>
     <row r="22" ht="15.75" customHeight="1"/>
     <row r="23" ht="15.75" customHeight="1"/>

</xml_diff>